<commit_message>
Let schedule breaks skip nomination and block, shown as interludes
The import forced a non-empty nomination and block on every row, so organizers had to invent placeholders (Вне конкурса, Открытие) for breaks, the opening and the closing — junk data to pass the validator, and stricter than the domain, which already models both as nullable and renders the fallback.

Read nomination_title and block_title as optional cells (title and duration stay required); leave them blank on the template's interlude rows and reorder the break between blocks. On the schedule page a block-less row is lifted out as a standalone dashed interlude row that stays interactive, and a block row with no nomination drops its sub-header.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/static/schedule-template.xlsx
+++ b/frontend/static/schedule-template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>number</t>
   </si>
@@ -34,12 +34,6 @@
     <t>Открытие фестиваля</t>
   </si>
   <si>
-    <t>Вне конкурса</t>
-  </si>
-  <si>
-    <t>Открытие</t>
-  </si>
-  <si>
     <t>Дефиле «Наруто»</t>
   </si>
   <si>
@@ -49,15 +43,15 @@
     <t>Косплей</t>
   </si>
   <si>
+    <t>Сценка «Стальной алхимик»</t>
+  </si>
+  <si>
+    <t>Групповое дефиле</t>
+  </si>
+  <si>
     <t>Перерыв</t>
   </si>
   <si>
-    <t>Сценка «Стальной алхимик»</t>
-  </si>
-  <si>
-    <t>Групповое дефиле</t>
-  </si>
-  <si>
     <t>Вокал: «Унесённые призраками»</t>
   </si>
   <si>
@@ -68,9 +62,6 @@
   </si>
   <si>
     <t>Награждение и закрытие</t>
-  </si>
-  <si>
-    <t>Закрытие</t>
   </si>
 </sst>
 </file>
@@ -461,102 +452,78 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="2">
         <v>900</v>
       </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" s="2">
         <v>45</v>
       </c>
       <c r="D3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
+      <c r="C4" s="2">
+        <v>480</v>
+      </c>
+      <c r="D4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="B4" t="s">
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C5" s="2">
         <v>600</v>
-      </c>
-      <c r="D4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="2">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2">
-        <v>480</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C6" s="2">
         <v>210</v>
       </c>
       <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="B7" t="s">
         <v>15</v>
-      </c>
-      <c r="E6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="2">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
       </c>
       <c r="C7" s="2">
         <v>1200</v>
-      </c>
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>